<commit_message>
Update CPI by category to show trends over time
Changed from single-month bar chart to multi-line time series showing
5 grouped spending categories from 2020-2025:
- Food & Dining
- Housing & Utilities
- Transport
- Services
- Other Goods

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/cpi-by-category-ulaanbaatar.xlsx
+++ b/data.mn/public/datasets/cpi-by-category-ulaanbaatar.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="November 2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPI by Category" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,153 +425,1359 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Change (%)</t>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Housing &amp; Utilities</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Other Goods</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Transport</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Recreation and culture</t>
+          <t>2020-02</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2666666666666666</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Miscellaneous goods and services</t>
+          <t>2020-03</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.2</v>
+        <v>1.666666666666667</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0333333333333333</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clothing, footwear and cloth</t>
+          <t>2020-04</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.9</v>
+        <v>0.6333333333333334</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-0.1333333333333333</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-2.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alcoholic beverages and tobacco</t>
+          <t>2020-05</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-2.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Furnishings, household equipment and tools</t>
+          <t>2020-06</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4</v>
+        <v>0.6999999999999998</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0666666666666666</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>2020-07</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0666666666666666</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F7" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Restaurants and hotels</t>
+          <t>2020-08</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.2</v>
+        <v>-1.533333333333333</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Health, medical care and services</t>
+          <t>2020-09</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.1</v>
+        <v>-0.8000000000000002</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.3666666666666667</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Food and non-alcaholic beverages</t>
+          <t>2020-10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Education services</t>
+          <t>2020-11</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>0.7333333333333334</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>2020-12</t>
         </is>
       </c>
       <c r="B12" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-4.933333333333334</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Insurance and financial services</t>
+          <t>2021-01</t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.3999999999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Housing, water, electricity and fuels</t>
+          <t>2021-02</t>
         </is>
       </c>
       <c r="B14" t="n">
+        <v>2.066666666666667</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2021-03</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1.533333333333333</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.1666666666666666</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2021-04</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2021-05</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1.066666666666667</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0666666666666666</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2021-06</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2021-07</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.0333333333333333</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F19" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2021-08</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>-0.3333333333333332</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2021-09</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2021-10</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.4666666666666666</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2.933333333333334</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.733333333333333</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2022-01</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1.933333333333334</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.975</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2022-02</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.4666666666666667</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.7666666666666666</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2022-03</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2022-04</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.366666666666666</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4.433333333333334</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2.025</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2.233333333333333</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.2666666666666666</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2022-06</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2.233333333333333</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.7666666666666666</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.7333333333333334</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>-0.8333333333333334</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3.025</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2022-09</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1.033333333333333</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.3249999999999999</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1.033333333333333</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.7666666666666666</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2022-12</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.3999999999999999</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.0499999999999999</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1.433333333333333</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.4666666666666666</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.7666666666666667</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2.533333333333333</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1.166666666666667</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.2249999999999999</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.9666666666666668</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>-0.0333333333333333</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.0333333333333333</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F43" t="n">
         <v>-0.7</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>-0.5333333333333332</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.0333333333333333</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E44" t="n">
+        <v>5.875</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.0666666666666666</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-0.2333333333333333</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1.133333333333333</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.7666666666666666</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.1666666666666666</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-1.3</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.2666666666666666</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>-0.1999999999999999</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.7333333333333334</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>-0.7666666666666666</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="D56" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E56" t="n">
+        <v>5.775</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.3666666666666667</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F57" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0.3666666666666667</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1.133333333333334</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4.600000000000001</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1.233333333333333</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.8000000000000002</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1.166666666666667</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E61" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>